<commit_message>
update test summary those 27 are fail
</commit_message>
<xml_diff>
--- a/test summary.xlsx
+++ b/test summary.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="244">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -293,7 +293,10 @@
 Thank you for shopping with us.
 Customer Rewards Department
 Retail Promotions &amp; Member Benefits
-ChatGPT can make mistakes. Check important info.</t>
+</t>
+  </si>
+  <si>
+    <t>spam</t>
   </si>
   <si>
     <t>security-alert@onlinebank-support.com</t>
@@ -1973,7 +1976,7 @@
         <v>18</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="G17" s="13">
         <v>0.12</v>
@@ -1991,13 +1994,13 @@
         <v>Test 016</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>13</v>
@@ -2006,13 +2009,13 @@
         <v>13</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2021,13 +2024,13 @@
         <v>Test 017</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E19" s="12" t="s">
         <v>13</v>
@@ -2036,10 +2039,10 @@
         <v>13</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I19" s="14" t="s">
         <v>14</v>
@@ -2051,13 +2054,13 @@
         <v>Test 018</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E20" s="12" t="s">
         <v>13</v>
@@ -2066,10 +2069,10 @@
         <v>13</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I20" s="14" t="s">
         <v>14</v>
@@ -2081,13 +2084,13 @@
         <v>Test 019</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E21" s="12" t="s">
         <v>13</v>
@@ -2096,10 +2099,10 @@
         <v>13</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I21" s="14" t="s">
         <v>14</v>
@@ -2111,25 +2114,25 @@
         <v>Test 020</v>
       </c>
       <c r="B22" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="C22" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="E22" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="12" t="s">
-        <v>77</v>
-      </c>
       <c r="H22" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I22" s="14" t="s">
         <v>14</v>
@@ -2141,13 +2144,13 @@
         <v>Test 021</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E23" s="12" t="s">
         <v>13</v>
@@ -2156,10 +2159,10 @@
         <v>13</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I23" s="14" t="s">
         <v>14</v>
@@ -2171,13 +2174,13 @@
         <v>Test 022</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E24" s="12" t="s">
         <v>13</v>
@@ -2186,13 +2189,13 @@
         <v>22</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="25" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2201,28 +2204,28 @@
         <v>Test 023</v>
       </c>
       <c r="B25" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="I25" s="14" t="s">
         <v>90</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="E25" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G25" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="I25" s="14" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="26" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2231,13 +2234,13 @@
         <v>Test 024</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E26" s="12" t="s">
         <v>13</v>
@@ -2246,13 +2249,13 @@
         <v>13</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2261,13 +2264,13 @@
         <v>Test 025</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E27" s="12" t="s">
         <v>13</v>
@@ -2276,13 +2279,13 @@
         <v>13</v>
       </c>
       <c r="G27" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H27" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2291,13 +2294,13 @@
         <v>Test 026</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E28" s="12" t="s">
         <v>13</v>
@@ -2306,13 +2309,13 @@
         <v>22</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="29" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2321,13 +2324,13 @@
         <v>Test 027</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E29" s="12" t="s">
         <v>13</v>
@@ -2336,13 +2339,13 @@
         <v>22</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2351,28 +2354,28 @@
         <v>Test 028</v>
       </c>
       <c r="B30" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G30" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="I30" s="14" t="s">
         <v>113</v>
-      </c>
-      <c r="C30" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="E30" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F30" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G30" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="H30" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="I30" s="14" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="31" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2381,13 +2384,13 @@
         <v>Test 029</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E31" s="12" t="s">
         <v>13</v>
@@ -2396,10 +2399,10 @@
         <v>22</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I31" s="14" t="s">
         <v>41</v>
@@ -2411,13 +2414,13 @@
         <v>Test 030</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E32" s="12" t="s">
         <v>13</v>
@@ -2426,10 +2429,10 @@
         <v>13</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I32" s="14" t="s">
         <v>14</v>
@@ -2441,13 +2444,13 @@
         <v>Test 031</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E33" s="12" t="s">
         <v>13</v>
@@ -2456,13 +2459,13 @@
         <v>22</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I33" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2471,13 +2474,13 @@
         <v>Test 032</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E34" s="12" t="s">
         <v>13</v>
@@ -2486,10 +2489,10 @@
         <v>22</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I34" s="14" t="s">
         <v>41</v>
@@ -2501,13 +2504,13 @@
         <v>Test 033</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E35" s="12" t="s">
         <v>13</v>
@@ -2516,10 +2519,10 @@
         <v>13</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H35" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I35" s="14" t="s">
         <v>14</v>
@@ -2531,13 +2534,13 @@
         <v>Test 034</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E36" s="12" t="s">
         <v>13</v>
@@ -2546,10 +2549,10 @@
         <v>22</v>
       </c>
       <c r="G36" s="12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I36" s="14" t="s">
         <v>41</v>
@@ -2561,13 +2564,13 @@
         <v>Test 035</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E37" s="12" t="s">
         <v>13</v>
@@ -2576,10 +2579,10 @@
         <v>13</v>
       </c>
       <c r="G37" s="12" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H37" s="12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I37" s="14" t="s">
         <v>14</v>
@@ -2591,13 +2594,13 @@
         <v>Test 036</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E38" s="12" t="s">
         <v>13</v>
@@ -2606,10 +2609,10 @@
         <v>22</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I38" s="14" t="s">
         <v>41</v>
@@ -2621,13 +2624,13 @@
         <v>Test 037</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E39" s="12" t="s">
         <v>13</v>
@@ -2636,10 +2639,10 @@
         <v>13</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I39" s="14" t="s">
         <v>14</v>
@@ -2651,13 +2654,13 @@
         <v>Test 038</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E40" s="12" t="s">
         <v>18</v>
@@ -2666,10 +2669,10 @@
         <v>22</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I40" s="14" t="s">
         <v>41</v>
@@ -2681,13 +2684,13 @@
         <v>Test 039</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E41" s="12" t="s">
         <v>18</v>
@@ -2696,10 +2699,10 @@
         <v>22</v>
       </c>
       <c r="G41" s="12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H41" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I41" s="14" t="s">
         <v>41</v>
@@ -2711,13 +2714,13 @@
         <v>Test 040</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E42" s="12" t="s">
         <v>18</v>
@@ -2726,10 +2729,10 @@
         <v>22</v>
       </c>
       <c r="G42" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H42" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I42" s="14" t="s">
         <v>41</v>
@@ -2741,13 +2744,13 @@
         <v>Test 041</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E43" s="12" t="s">
         <v>18</v>
@@ -2756,10 +2759,10 @@
         <v>22</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I43" s="14" t="s">
         <v>41</v>
@@ -2771,13 +2774,13 @@
         <v>Test 042</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E44" s="12" t="s">
         <v>13</v>
@@ -2786,10 +2789,10 @@
         <v>22</v>
       </c>
       <c r="G44" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I44" s="14" t="s">
         <v>41</v>
@@ -2801,13 +2804,13 @@
         <v>Test 043</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E45" s="12" t="s">
         <v>13</v>
@@ -2816,10 +2819,10 @@
         <v>22</v>
       </c>
       <c r="G45" s="12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I45" s="14" t="s">
         <v>41</v>
@@ -2831,28 +2834,28 @@
         <v>Test 044</v>
       </c>
       <c r="B46" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="D46" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G46" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="H46" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="C46" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="D46" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="E46" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F46" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G46" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="H46" s="12" t="s">
-        <v>175</v>
-      </c>
       <c r="I46" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2861,13 +2864,13 @@
         <v>Test 045</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E47" s="12" t="s">
         <v>13</v>
@@ -2876,10 +2879,10 @@
         <v>22</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H47" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I47" s="14" t="s">
         <v>41</v>
@@ -2891,13 +2894,13 @@
         <v>Test 046</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E48" s="12" t="s">
         <v>22</v>
@@ -2906,10 +2909,10 @@
         <v>22</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H48" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I48" s="14" t="s">
         <v>14</v>
@@ -2921,13 +2924,13 @@
         <v>Test 047</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E49" s="12" t="s">
         <v>22</v>
@@ -2936,10 +2939,10 @@
         <v>22</v>
       </c>
       <c r="G49" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H49" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I49" s="14" t="s">
         <v>14</v>
@@ -2951,13 +2954,13 @@
         <v>Test 048</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E50" s="12" t="s">
         <v>22</v>
@@ -2966,10 +2969,10 @@
         <v>22</v>
       </c>
       <c r="G50" s="12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H50" s="12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I50" s="14" t="s">
         <v>14</v>
@@ -2981,13 +2984,13 @@
         <v>Test 049</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E51" s="12" t="s">
         <v>22</v>
@@ -2996,10 +2999,10 @@
         <v>22</v>
       </c>
       <c r="G51" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H51" s="12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I51" s="14" t="s">
         <v>14</v>
@@ -3011,13 +3014,13 @@
         <v>Test 050</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E52" s="12" t="s">
         <v>22</v>
@@ -3026,10 +3029,10 @@
         <v>22</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I52" s="14" t="s">
         <v>14</v>
@@ -3041,13 +3044,13 @@
         <v>Test 051</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E53" s="12" t="s">
         <v>22</v>
@@ -3056,10 +3059,10 @@
         <v>22</v>
       </c>
       <c r="G53" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H53" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I53" s="14" t="s">
         <v>14</v>
@@ -3071,13 +3074,13 @@
         <v>Test 052</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E54" s="12" t="s">
         <v>22</v>
@@ -3086,10 +3089,10 @@
         <v>22</v>
       </c>
       <c r="G54" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H54" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I54" s="14" t="s">
         <v>14</v>
@@ -3101,13 +3104,13 @@
         <v>Test 053</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E55" s="12" t="s">
         <v>22</v>
@@ -3116,10 +3119,10 @@
         <v>22</v>
       </c>
       <c r="G55" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H55" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I55" s="14" t="s">
         <v>14</v>
@@ -3131,13 +3134,13 @@
         <v>Test 054</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E56" s="12" t="s">
         <v>22</v>
@@ -3146,10 +3149,10 @@
         <v>22</v>
       </c>
       <c r="G56" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H56" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I56" s="14" t="s">
         <v>14</v>
@@ -3161,13 +3164,13 @@
         <v>Test 055</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E57" s="12" t="s">
         <v>22</v>
@@ -3176,10 +3179,10 @@
         <v>22</v>
       </c>
       <c r="G57" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H57" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I57" s="14" t="s">
         <v>14</v>
@@ -3191,13 +3194,13 @@
         <v>Test 056</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E58" s="12" t="s">
         <v>18</v>
@@ -3206,10 +3209,10 @@
         <v>22</v>
       </c>
       <c r="G58" s="12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H58" s="12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I58" s="14" t="s">
         <v>41</v>
@@ -3221,13 +3224,13 @@
         <v>Test 057</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E59" s="12" t="s">
         <v>18</v>
@@ -3236,10 +3239,10 @@
         <v>18</v>
       </c>
       <c r="G59" s="12" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H59" s="12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I59" s="14" t="s">
         <v>14</v>
@@ -3251,13 +3254,13 @@
         <v>Test 058</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D60" s="11" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E60" s="12" t="s">
         <v>18</v>
@@ -3266,13 +3269,13 @@
         <v>22</v>
       </c>
       <c r="G60" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H60" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I60" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="61" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3281,13 +3284,13 @@
         <v>Test 059</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D61" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E61" s="12" t="s">
         <v>18</v>
@@ -3296,13 +3299,13 @@
         <v>22</v>
       </c>
       <c r="G61" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H61" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I61" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="62" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3311,13 +3314,13 @@
         <v>Test 060</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D62" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E62" s="12" t="s">
         <v>18</v>
@@ -3326,10 +3329,10 @@
         <v>22</v>
       </c>
       <c r="G62" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H62" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I62" s="14" t="s">
         <v>41</v>
@@ -3341,13 +3344,13 @@
         <v>Test 061</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E63" s="12" t="s">
         <v>13</v>
@@ -3356,10 +3359,10 @@
         <v>22</v>
       </c>
       <c r="G63" s="12" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H63" s="12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I63" s="14" t="s">
         <v>41</v>
@@ -3371,13 +3374,13 @@
         <v>Test 062</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E64" s="12" t="s">
         <v>13</v>
@@ -3386,10 +3389,10 @@
         <v>22</v>
       </c>
       <c r="G64" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H64" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I64" s="14" t="s">
         <v>41</v>
@@ -3401,13 +3404,13 @@
         <v>Test 063</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E65" s="12" t="s">
         <v>22</v>
@@ -3416,10 +3419,10 @@
         <v>22</v>
       </c>
       <c r="G65" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H65" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I65" s="14" t="s">
         <v>14</v>
@@ -3431,13 +3434,13 @@
         <v>Test 064</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E66" s="12" t="s">
         <v>22</v>
@@ -3446,10 +3449,10 @@
         <v>22</v>
       </c>
       <c r="G66" s="12" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I66" s="14" t="s">
         <v>14</v>
@@ -3461,13 +3464,13 @@
         <v>Test 065</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E67" s="12" t="s">
         <v>13</v>
@@ -3476,13 +3479,13 @@
         <v>22</v>
       </c>
       <c r="G67" s="12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H67" s="12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I67" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="68" ht="21" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>